<commit_message>
fix: resolve orphaned policy repo IDs in extractor
- Policies pointing at deleted repos now labeled '(deleted repo)' instead of '?'
- Attempt direct repo API fetch before giving up
- Project-wide policies only auto-target live repos, not deleted ones
- Deleted-repo policies indicate ADO-side stale config to clean up pre-migration
</commit_message>
<xml_diff>
--- a/Documents/ADO Inventory zeb-ai.xlsx
+++ b/Documents/ADO Inventory zeb-ai.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08 17:33 UTC</t>
+          <t>2026-07-08 17:49 UTC</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>(deleted repo)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -4731,7 +4731,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>(deleted repo)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -4971,7 +4971,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>(deleted repo)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>(deleted repo)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">

</xml_diff>